<commit_message>
Middle tier for an added student's cost; share card; FY2026 Circuit Breaker fix
- scripts/special_education_cost_per_student.py: open seat plus special
  education at the district average (DESE FY2025, net of grants and the
  FY2026 Circuit Breaker payment, with benefits), about $7,760 in FY2027 dollars
- data/dese_sped/: DESE special education spending and Circuit Breaker files
- Schools page: three tiers for the cost of an added student
- Share card for link previews
- Circuit Breaker correction to the open-seat cost range

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KdZ1NChRRYkpsgRG6uA8od
</commit_message>
<xml_diff>
--- a/Brookline_Enrollment_Explained.xlsx
+++ b/Brookline_Enrollment_Explained.xlsx
@@ -240,12 +240,12 @@
     </comment>
     <comment ref="G27" authorId="0" shapeId="0">
       <text>
-        <t>September 2026: K-8 derived from the Superintendent's class-size table (average x sections); 9-12 and BEEP as reported. Approximate to within a student or two per grade.</t>
+        <t>October 1, 2026 (SIMS submission to DESE), as reported by the School Department; the 11 ungraded high school students are in the total but not in a grade.</t>
       </text>
     </comment>
     <comment ref="I27" authorId="0" shapeId="0">
       <text>
-        <t>School Department, September 2026 count</t>
+        <t>School Department, October 1, 2026 count</t>
       </text>
     </comment>
   </commentList>
@@ -260,7 +260,7 @@
   <commentList>
     <comment ref="K10" authorId="0" shapeId="0">
       <text>
-        <t>September 2026: K-8 derived from the Superintendent's class-size table (average x sections); 9-12 and BEEP as reported. Approximate to within a student or two per grade.</t>
+        <t>October 1, 2026 (SIMS submission to DESE), as reported by the School Department; the 11 ungraded high school students are in the total but not in a grade.</t>
       </text>
     </comment>
   </commentList>
@@ -300,7 +300,7 @@
   <commentList>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
-        <t>September 2026: K-8 derived from the Superintendent's class-size table (average x sections); 9-12 and BEEP as reported. Approximate to within a student or two per grade.</t>
+        <t>October 1, 2026 (SIMS submission to DESE), as reported by the School Department; the 11 ungraded high school students are in the total but not in a grade.</t>
       </text>
     </comment>
   </commentList>
@@ -2257,14 +2257,14 @@
         <v/>
       </c>
       <c r="G27" s="12" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="H27" s="13">
         <f>G27/E27</f>
         <v/>
       </c>
       <c r="I27" s="12" t="n">
-        <v>6889</v>
+        <v>6833</v>
       </c>
       <c r="J27" s="13">
         <f>I27/F27</f>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="O27" s="11" t="n"/>
       <c r="P27" s="12" t="n">
-        <v>6889</v>
+        <v>6833</v>
       </c>
       <c r="Q27" s="13">
         <f>P27/F27</f>
@@ -2363,10 +2363,10 @@
         <v/>
       </c>
       <c r="O28" s="12" t="n">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="P28" s="12" t="n">
-        <v>6716</v>
+        <v>6662</v>
       </c>
       <c r="Q28" s="13">
         <f>P28/F28</f>
@@ -2444,10 +2444,10 @@
         <v/>
       </c>
       <c r="O29" s="12" t="n">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="P29" s="12" t="n">
-        <v>6554</v>
+        <v>6501</v>
       </c>
       <c r="Q29" s="13">
         <f>P29/F29</f>
@@ -2525,10 +2525,10 @@
         <v/>
       </c>
       <c r="O30" s="12" t="n">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="P30" s="12" t="n">
-        <v>6455</v>
+        <v>6402</v>
       </c>
       <c r="Q30" s="13">
         <f>P30/F30</f>
@@ -2606,10 +2606,10 @@
         <v/>
       </c>
       <c r="O31" s="12" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="P31" s="12" t="n">
-        <v>6313</v>
+        <v>6262</v>
       </c>
       <c r="Q31" s="13">
         <f>P31/F31</f>
@@ -2687,10 +2687,10 @@
         <v/>
       </c>
       <c r="O32" s="12" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="P32" s="12" t="n">
-        <v>6222</v>
+        <v>6171</v>
       </c>
       <c r="Q32" s="13">
         <f>P32/F32</f>
@@ -2768,10 +2768,10 @@
         <v/>
       </c>
       <c r="O33" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P33" s="12" t="n">
-        <v>6104</v>
+        <v>6054</v>
       </c>
       <c r="Q33" s="13">
         <f>P33/F33</f>
@@ -2849,10 +2849,10 @@
         <v/>
       </c>
       <c r="O34" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P34" s="12" t="n">
-        <v>5975</v>
+        <v>5926</v>
       </c>
       <c r="Q34" s="13">
         <f>P34/F34</f>
@@ -2921,10 +2921,10 @@
       <c r="M35" s="11" t="n"/>
       <c r="N35" s="11" t="n"/>
       <c r="O35" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P35" s="12" t="n">
-        <v>5854</v>
+        <v>5806</v>
       </c>
       <c r="Q35" s="13">
         <f>P35/F35</f>
@@ -2983,10 +2983,10 @@
       <c r="M36" s="11" t="n"/>
       <c r="N36" s="11" t="n"/>
       <c r="O36" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P36" s="12" t="n">
-        <v>5726</v>
+        <v>5680</v>
       </c>
       <c r="Q36" s="13">
         <f>P36/F36</f>
@@ -3045,10 +3045,10 @@
       <c r="M37" s="11" t="n"/>
       <c r="N37" s="11" t="n"/>
       <c r="O37" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P37" s="12" t="n">
-        <v>5630</v>
+        <v>5584</v>
       </c>
       <c r="Q37" s="13">
         <f>P37/F37</f>
@@ -3107,10 +3107,10 @@
       <c r="M38" s="11" t="n"/>
       <c r="N38" s="11" t="n"/>
       <c r="O38" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P38" s="12" t="n">
-        <v>5514</v>
+        <v>5469</v>
       </c>
       <c r="Q38" s="13">
         <f>P38/F38</f>
@@ -3169,10 +3169,10 @@
       <c r="M39" s="11" t="n"/>
       <c r="N39" s="11" t="n"/>
       <c r="O39" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P39" s="12" t="n">
-        <v>5480</v>
+        <v>5435</v>
       </c>
       <c r="Q39" s="13">
         <f>P39/F39</f>
@@ -3231,10 +3231,10 @@
       <c r="M40" s="11" t="n"/>
       <c r="N40" s="11" t="n"/>
       <c r="O40" s="12" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="P40" s="12" t="n">
-        <v>5444</v>
+        <v>5400</v>
       </c>
       <c r="Q40" s="13">
         <f>P40/F40</f>
@@ -3331,14 +3331,14 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>So 415 becomes 415 x 1.029 = 427 in grade 1, then 427 x 1.023 = 437 in grade 2, and so on. The 'Change' columns show each year's ratio. The base case follows the same steps, from NESDEC's numbers scaled up 1.7% to match the September 2026 count (2021 births were already counted, so this class needs no births adjustment).</t>
+          <t>So 415 becomes 415 x 1.029 = 427 in grade 1, then 427 x 1.023 = 437 in grade 2, and so on. The 'Change' columns show each year's ratio. The base case follows the same steps, from NESDEC's numbers scaled up 1.7% to match the October 1, 2026 count (2021 births were already counted, so this class needs no births adjustment).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>The School Department's forecast starts the same class at 507 and keeps it growing: its ratios assume more families moving in at every age. The actual kindergarten in September 2026 was about 411.</t>
+          <t>The School Department's forecast starts the same class at 507 and keeps it growing: its ratios assume more families moving in at every age. The actual kindergarten on October 1, 2026 was 410.</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3419,7 @@
         <v>415</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>507</v>
@@ -3429,7 +3429,7 @@
         <v/>
       </c>
       <c r="K10" s="15" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11">
@@ -3456,7 +3456,7 @@
         <v/>
       </c>
       <c r="F11" s="15" t="n">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="G11" s="17">
         <f>IF(AND(ISNUMBER(F11),ISNUMBER(F10)),F11/F10,"")</f>
@@ -3498,7 +3498,7 @@
         <v/>
       </c>
       <c r="F12" s="15" t="n">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="G12" s="17">
         <f>IF(AND(ISNUMBER(F12),ISNUMBER(F11)),F12/F11,"")</f>
@@ -3540,7 +3540,7 @@
         <v/>
       </c>
       <c r="F13" s="15" t="n">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="G13" s="17">
         <f>IF(AND(ISNUMBER(F13),ISNUMBER(F12)),F13/F12,"")</f>
@@ -3582,7 +3582,7 @@
         <v/>
       </c>
       <c r="F14" s="15" t="n">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="G14" s="17">
         <f>IF(AND(ISNUMBER(F14),ISNUMBER(F13)),F14/F13,"")</f>
@@ -3624,7 +3624,7 @@
         <v/>
       </c>
       <c r="F15" s="15" t="n">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="G15" s="17">
         <f>IF(AND(ISNUMBER(F15),ISNUMBER(F14)),F15/F14,"")</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="F16" s="15" t="n">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="G16" s="17">
         <f>IF(AND(ISNUMBER(F16),ISNUMBER(F15)),F16/F15,"")</f>
@@ -3708,7 +3708,7 @@
         <v/>
       </c>
       <c r="F17" s="15" t="n">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="G17" s="17">
         <f>IF(AND(ISNUMBER(F17),ISNUMBER(F16)),F17/F16,"")</f>
@@ -3747,7 +3747,7 @@
         <v/>
       </c>
       <c r="F18" s="15" t="n">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="G18" s="17">
         <f>IF(AND(ISNUMBER(F18),ISNUMBER(F17)),F18/F17,"")</f>
@@ -3783,7 +3783,7 @@
         <v/>
       </c>
       <c r="F19" s="15" t="n">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="G19" s="17">
         <f>IF(AND(ISNUMBER(F19),ISNUMBER(F18)),F19/F18,"")</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="F20" s="15" t="n">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="G20" s="17">
         <f>IF(AND(ISNUMBER(F20),ISNUMBER(F19)),F20/F19,"")</f>
@@ -3855,7 +3855,7 @@
         <v/>
       </c>
       <c r="F21" s="15" t="n">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="G21" s="17">
         <f>IF(AND(ISNUMBER(F21),ISNUMBER(F20)),F21/F20,"")</f>
@@ -3891,7 +3891,7 @@
         <v/>
       </c>
       <c r="F22" s="15" t="n">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="G22" s="17">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER(F21)),F22/F21,"")</f>
@@ -3909,7 +3909,7 @@
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>Kindergarten row: NESDEC's 415 = 491 births x 0.845. Your scenario's kindergarten starts from the September 2026 count (about 411) and follows the ratios on Inputs. Past FY2034 only the base case and Your scenario continue; the base case extends NESDEC's table with its average ratios.</t>
+          <t>Kindergarten row: NESDEC's 415 = 491 births x 0.845. Your scenario's kindergarten starts from the October 1, 2026 count (410) and follows the ratios on Inputs. Past FY2034 only the base case and Your scenario continue; the base case extends NESDEC's table with its average ratios.</t>
         </is>
       </c>
     </row>
@@ -5120,7 +5120,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Your scenario: a live cohort model from the September 2026 (FY2027) actual grades</t>
+          <t>Your scenario: a live cohort model from the October 1, 2026 (FY2027) actual grades</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="C6" s="25">
         <f>Inputs!$B$5</f>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="B7" s="15" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C7" s="25">
         <f>INDEX(Inputs!$B$26:$B$80,MATCH(C$5,Inputs!$A$26:$A$80,0))*Inputs!$B$4</f>
@@ -5388,7 +5388,7 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C8" s="25">
         <f>B7*Inputs!$B$9</f>
@@ -5450,7 +5450,7 @@
         </is>
       </c>
       <c r="B9" s="15" t="n">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="C9" s="25">
         <f>B8*Inputs!$B$10</f>
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C10" s="25">
         <f>B9*Inputs!$B$11</f>
@@ -5574,7 +5574,7 @@
         </is>
       </c>
       <c r="B11" s="15" t="n">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C11" s="25">
         <f>B10*Inputs!$B$12</f>
@@ -5636,7 +5636,7 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="C12" s="25">
         <f>B11*Inputs!$B$13</f>
@@ -5698,7 +5698,7 @@
         </is>
       </c>
       <c r="B13" s="15" t="n">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="C13" s="25">
         <f>B12*Inputs!$B$14</f>
@@ -5760,7 +5760,7 @@
         </is>
       </c>
       <c r="B14" s="15" t="n">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="C14" s="25">
         <f>B13*Inputs!$B$15</f>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="B15" s="15" t="n">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="C15" s="25">
         <f>B14*Inputs!$B$16</f>
@@ -5884,7 +5884,7 @@
         </is>
       </c>
       <c r="B16" s="15" t="n">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C16" s="25">
         <f>B15*Inputs!$B$17</f>
@@ -5946,7 +5946,7 @@
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="C17" s="25">
         <f>B16*Inputs!$B$18</f>
@@ -6008,7 +6008,7 @@
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C18" s="25">
         <f>B17*Inputs!$B$19</f>
@@ -6070,7 +6070,7 @@
         </is>
       </c>
       <c r="B19" s="15" t="n">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="C19" s="25">
         <f>B18*Inputs!$B$20</f>
@@ -6202,46 +6202,46 @@
         </is>
       </c>
       <c r="B23" s="25" t="n">
-        <v>6889</v>
+        <v>6833</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>6716</v>
+        <v>6662</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>6554</v>
+        <v>6501</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>6455</v>
+        <v>6402</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>6313</v>
+        <v>6262</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>6222</v>
+        <v>6171</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>6104</v>
+        <v>6054</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>5975</v>
+        <v>5926</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>5854</v>
+        <v>5806</v>
       </c>
       <c r="K23" s="25" t="n">
-        <v>5726</v>
+        <v>5680</v>
       </c>
       <c r="L23" s="25" t="n">
-        <v>5630</v>
+        <v>5584</v>
       </c>
       <c r="M23" s="25" t="n">
-        <v>5514</v>
+        <v>5469</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>5480</v>
+        <v>5435</v>
       </c>
       <c r="O23" s="25" t="n">
-        <v>5444</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="24">
@@ -6309,7 +6309,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Why this differs a little from the base case: the base case runs NESDEC's own grade table (adjusted for actual births), scales it to the September 2026 count and adds the children of the Chestnut Hill homes; this sheet starts from the September 2026 grades and applies the ratios directly. The September 2026 grades sum to 6,875 (the reported 6,889 also counts 11 special-program students and rounding).</t>
+          <t>Why this differs a little from the base case: the base case runs NESDEC's own grade table (adjusted for actual births), scales it to the October 1, 2026 count and adds the children of the Chestnut Hill homes; this sheet starts from the October 1, 2026 grades and applies the ratios directly. The October 1, 2026 grades sum to 6,822 (the reported 6,833 also counts 11 ungraded high school students).</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6363,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>FY2014-FY2024 from NESDEC's historical table; FY2025-FY2026 from DESE; FY2027 from the Superintendent's September 2026 class-size table (approximate). Excludes ungraded and special-program students.</t>
+          <t>FY2014-FY2024 from NESDEC's historical table; FY2025-FY2026 from DESE; FY2027 from the School Department's October 1, 2026 count. Excludes ungraded and special-program students.</t>
         </is>
       </c>
     </row>
@@ -7145,46 +7145,46 @@
         </is>
       </c>
       <c r="B19" s="15" t="n">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="C19" s="15" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="I19" s="15" t="n">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="J19" s="15" t="n">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="K19" s="15" t="n">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="L19" s="15" t="n">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="M19" s="15" t="n">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="N19" s="15" t="n">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="O19" s="15" t="n">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="P19" s="27">
         <f>SUM(B19:O19)</f>
@@ -7873,14 +7873,14 @@
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>Base case: NESDEC adjusted for actual births, scaled to the September 2026 count</t>
+          <t>Base case: NESDEC adjusted for actual births, scaled to the October 1, 2026 count</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Each class born 2022 or later scaled by actual / NESDEC births (2022: 482/459; 2023: 422/518; 2024: 443/507; 2025 on: the 2022-24 average, 449 a year); extended past FY2034 with NESDEC's average ratios; all x 1.017 so FY2027 matches 6,889. The model also adds about 30 children from the Chestnut Hill homes, not shown by grade.</t>
+          <t>Each class born 2022 or later scaled by actual / NESDEC births (2022: 482/459; 2023: 422/518; 2024: 443/507; 2025 on: the 2022-24 average, 449 a year); extended past FY2034 with NESDEC's average ratios; all x 1.009 so FY2027 matches 6,833. The model also adds about 30 children from the Chestnut Hill homes, not shown by grade.</t>
         </is>
       </c>
     </row>
@@ -7973,46 +7973,46 @@
         </is>
       </c>
       <c r="B39" s="15" t="n">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C39" s="15" t="n">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="D39" s="15" t="n">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="E39" s="15" t="n">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="F39" s="15" t="n">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="G39" s="15" t="n">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="I39" s="15" t="n">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="J39" s="15" t="n">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="K39" s="15" t="n">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="L39" s="15" t="n">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="M39" s="15" t="n">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="N39" s="15" t="n">
-        <v>560</v>
+        <v>556</v>
       </c>
       <c r="O39" s="15" t="n">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="P39" s="27">
         <f>SUM(B39:O39)</f>
@@ -8026,46 +8026,46 @@
         </is>
       </c>
       <c r="B40" s="15" t="n">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C40" s="15" t="n">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="D40" s="15" t="n">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="F40" s="15" t="n">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="G40" s="15" t="n">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="I40" s="15" t="n">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="J40" s="15" t="n">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="K40" s="15" t="n">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="M40" s="15" t="n">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="N40" s="15" t="n">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="O40" s="15" t="n">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="P40" s="27">
         <f>SUM(B40:O40)</f>
@@ -8079,46 +8079,46 @@
         </is>
       </c>
       <c r="B41" s="15" t="n">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C41" s="15" t="n">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="D41" s="15" t="n">
+        <v>510</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>502</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>537</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>537</v>
+      </c>
+      <c r="H41" s="15" t="n">
+        <v>554</v>
+      </c>
+      <c r="I41" s="15" t="n">
         <v>515</v>
       </c>
-      <c r="E41" s="15" t="n">
-        <v>506</v>
-      </c>
-      <c r="F41" s="15" t="n">
-        <v>541</v>
-      </c>
-      <c r="G41" s="15" t="n">
-        <v>541</v>
-      </c>
-      <c r="H41" s="15" t="n">
-        <v>558</v>
-      </c>
-      <c r="I41" s="15" t="n">
-        <v>520</v>
-      </c>
       <c r="J41" s="15" t="n">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="K41" s="15" t="n">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="L41" s="15" t="n">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="M41" s="15" t="n">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="N41" s="15" t="n">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="O41" s="15" t="n">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="P41" s="27">
         <f>SUM(B41:O41)</f>
@@ -8132,46 +8132,46 @@
         </is>
       </c>
       <c r="B42" s="15" t="n">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C42" s="15" t="n">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="D42" s="15" t="n">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="E42" s="15" t="n">
+        <v>523</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>502</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>542</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <v>537</v>
+      </c>
+      <c r="I42" s="15" t="n">
         <v>527</v>
       </c>
-      <c r="F42" s="15" t="n">
-        <v>506</v>
-      </c>
-      <c r="G42" s="15" t="n">
-        <v>546</v>
-      </c>
-      <c r="H42" s="15" t="n">
-        <v>541</v>
-      </c>
-      <c r="I42" s="15" t="n">
-        <v>531</v>
-      </c>
       <c r="J42" s="15" t="n">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="K42" s="15" t="n">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="M42" s="15" t="n">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="N42" s="15" t="n">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="O42" s="15" t="n">
-        <v>592</v>
+        <v>587</v>
       </c>
       <c r="P42" s="27">
         <f>SUM(B42:O42)</f>
@@ -8185,46 +8185,46 @@
         </is>
       </c>
       <c r="B43" s="15" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C43" s="15" t="n">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="D43" s="15" t="n">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="E43" s="15" t="n">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F43" s="15" t="n">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="G43" s="15" t="n">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="I43" s="15" t="n">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="J43" s="15" t="n">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="K43" s="15" t="n">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="L43" s="15" t="n">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="M43" s="15" t="n">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N43" s="15" t="n">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="O43" s="15" t="n">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="P43" s="27">
         <f>SUM(B43:O43)</f>
@@ -8238,46 +8238,46 @@
         </is>
       </c>
       <c r="B44" s="15" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C44" s="15" t="n">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D44" s="15" t="n">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G44" s="15" t="n">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="I44" s="15" t="n">
+        <v>515</v>
+      </c>
+      <c r="J44" s="15" t="n">
+        <v>507</v>
+      </c>
+      <c r="K44" s="15" t="n">
         <v>520</v>
       </c>
-      <c r="J44" s="15" t="n">
-        <v>512</v>
-      </c>
-      <c r="K44" s="15" t="n">
-        <v>525</v>
-      </c>
       <c r="L44" s="15" t="n">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="M44" s="15" t="n">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="N44" s="15" t="n">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O44" s="15" t="n">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="P44" s="27">
         <f>SUM(B44:O44)</f>
@@ -8291,46 +8291,46 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C45" s="15" t="n">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="D45" s="15" t="n">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E45" s="15" t="n">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="F45" s="15" t="n">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="G45" s="15" t="n">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="I45" s="15" t="n">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="J45" s="15" t="n">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="K45" s="15" t="n">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="L45" s="15" t="n">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="M45" s="15" t="n">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="N45" s="15" t="n">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="O45" s="15" t="n">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="P45" s="27">
         <f>SUM(B45:O45)</f>
@@ -8344,46 +8344,46 @@
         </is>
       </c>
       <c r="B46" s="15" t="n">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C46" s="15" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="D46" s="15" t="n">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="F46" s="15" t="n">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="G46" s="15" t="n">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="I46" s="15" t="n">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="J46" s="15" t="n">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="K46" s="15" t="n">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="M46" s="15" t="n">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="N46" s="15" t="n">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="O46" s="15" t="n">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="P46" s="27">
         <f>SUM(B46:O46)</f>
@@ -8397,46 +8397,46 @@
         </is>
       </c>
       <c r="B47" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C47" s="15" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="D47" s="15" t="n">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E47" s="15" t="n">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="F47" s="15" t="n">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="G47" s="15" t="n">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="I47" s="15" t="n">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="J47" s="15" t="n">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="K47" s="15" t="n">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="L47" s="15" t="n">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="M47" s="15" t="n">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="N47" s="15" t="n">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="O47" s="15" t="n">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="P47" s="27">
         <f>SUM(B47:O47)</f>
@@ -8450,46 +8450,46 @@
         </is>
       </c>
       <c r="B48" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C48" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D48" s="15" t="n">
+        <v>395</v>
+      </c>
+      <c r="E48" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="F48" s="15" t="n">
         <v>399</v>
       </c>
-      <c r="E48" s="15" t="n">
-        <v>407</v>
-      </c>
-      <c r="F48" s="15" t="n">
-        <v>403</v>
-      </c>
       <c r="G48" s="15" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="I48" s="15" t="n">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="J48" s="15" t="n">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="K48" s="15" t="n">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="M48" s="15" t="n">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="N48" s="15" t="n">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="O48" s="15" t="n">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="P48" s="27">
         <f>SUM(B48:O48)</f>
@@ -8503,46 +8503,46 @@
         </is>
       </c>
       <c r="B49" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C49" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D49" s="15" t="n">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E49" s="15" t="n">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="F49" s="15" t="n">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="G49" s="15" t="n">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="I49" s="15" t="n">
+        <v>418</v>
+      </c>
+      <c r="J49" s="15" t="n">
         <v>421</v>
       </c>
-      <c r="J49" s="15" t="n">
-        <v>424</v>
-      </c>
       <c r="K49" s="15" t="n">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="L49" s="15" t="n">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="M49" s="15" t="n">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="N49" s="15" t="n">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="O49" s="15" t="n">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="P49" s="27">
         <f>SUM(B49:O49)</f>
@@ -8556,46 +8556,46 @@
         </is>
       </c>
       <c r="B50" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C50" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D50" s="15" t="n">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E50" s="15" t="n">
+        <v>404</v>
+      </c>
+      <c r="F50" s="15" t="n">
+        <v>404</v>
+      </c>
+      <c r="G50" s="15" t="n">
         <v>407</v>
       </c>
-      <c r="F50" s="15" t="n">
-        <v>408</v>
-      </c>
-      <c r="G50" s="15" t="n">
-        <v>411</v>
-      </c>
       <c r="H50" s="15" t="n">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="I50" s="15" t="n">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="J50" s="15" t="n">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="K50" s="15" t="n">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="M50" s="15" t="n">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="N50" s="15" t="n">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="O50" s="15" t="n">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="P50" s="27">
         <f>SUM(B50:O50)</f>
@@ -8609,46 +8609,46 @@
         </is>
       </c>
       <c r="B51" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C51" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D51" s="15" t="n">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E51" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="F51" s="15" t="n">
+        <v>404</v>
+      </c>
+      <c r="G51" s="15" t="n">
+        <v>408</v>
+      </c>
+      <c r="H51" s="15" t="n">
         <v>407</v>
       </c>
-      <c r="F51" s="15" t="n">
-        <v>407</v>
-      </c>
-      <c r="G51" s="15" t="n">
-        <v>412</v>
-      </c>
-      <c r="H51" s="15" t="n">
-        <v>411</v>
-      </c>
       <c r="I51" s="15" t="n">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="J51" s="15" t="n">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="K51" s="15" t="n">
+        <v>413</v>
+      </c>
+      <c r="L51" s="15" t="n">
         <v>417</v>
       </c>
-      <c r="L51" s="15" t="n">
+      <c r="M51" s="15" t="n">
         <v>420</v>
       </c>
-      <c r="M51" s="15" t="n">
-        <v>423</v>
-      </c>
       <c r="N51" s="15" t="n">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="O51" s="15" t="n">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="P51" s="27">
         <f>SUM(B51:O51)</f>
@@ -8662,46 +8662,46 @@
         </is>
       </c>
       <c r="B52" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C52" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D52" s="15" t="n">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="F52" s="15" t="n">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="G52" s="15" t="n">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="H52" s="15" t="n">
+        <v>408</v>
+      </c>
+      <c r="I52" s="15" t="n">
+        <v>387</v>
+      </c>
+      <c r="J52" s="15" t="n">
+        <v>382</v>
+      </c>
+      <c r="K52" s="15" t="n">
+        <v>361</v>
+      </c>
+      <c r="L52" s="15" t="n">
         <v>412</v>
       </c>
-      <c r="I52" s="15" t="n">
-        <v>391</v>
-      </c>
-      <c r="J52" s="15" t="n">
-        <v>385</v>
-      </c>
-      <c r="K52" s="15" t="n">
-        <v>364</v>
-      </c>
-      <c r="L52" s="15" t="n">
-        <v>415</v>
-      </c>
       <c r="M52" s="15" t="n">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="N52" s="15" t="n">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="O52" s="15" t="n">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="P52" s="27">
         <f>SUM(B52:O52)</f>
@@ -8715,46 +8715,46 @@
         </is>
       </c>
       <c r="B53" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C53" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D53" s="15" t="n">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E53" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="F53" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="G53" s="15" t="n">
         <v>407</v>
       </c>
-      <c r="F53" s="15" t="n">
-        <v>407</v>
-      </c>
-      <c r="G53" s="15" t="n">
-        <v>410</v>
-      </c>
       <c r="H53" s="15" t="n">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="I53" s="15" t="n">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="J53" s="15" t="n">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="K53" s="15" t="n">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="L53" s="15" t="n">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="M53" s="15" t="n">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="N53" s="15" t="n">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="O53" s="15" t="n">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="P53" s="27">
         <f>SUM(B53:O53)</f>
@@ -8768,46 +8768,46 @@
         </is>
       </c>
       <c r="B54" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C54" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D54" s="15" t="n">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E54" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="F54" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="G54" s="15" t="n">
         <v>407</v>
       </c>
-      <c r="F54" s="15" t="n">
+      <c r="H54" s="15" t="n">
         <v>407</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>410</v>
-      </c>
-      <c r="H54" s="15" t="n">
-        <v>410</v>
-      </c>
       <c r="I54" s="15" t="n">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="J54" s="15" t="n">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="K54" s="15" t="n">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="M54" s="15" t="n">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="N54" s="15" t="n">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="O54" s="15" t="n">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="P54" s="27">
         <f>SUM(B54:O54)</f>
@@ -8821,46 +8821,46 @@
         </is>
       </c>
       <c r="B55" s="15" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C55" s="15" t="n">
+        <v>382</v>
+      </c>
+      <c r="D55" s="15" t="n">
+        <v>394</v>
+      </c>
+      <c r="E55" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="F55" s="15" t="n">
+        <v>403</v>
+      </c>
+      <c r="G55" s="15" t="n">
+        <v>407</v>
+      </c>
+      <c r="H55" s="15" t="n">
+        <v>407</v>
+      </c>
+      <c r="I55" s="15" t="n">
+        <v>387</v>
+      </c>
+      <c r="J55" s="15" t="n">
+        <v>386</v>
+      </c>
+      <c r="K55" s="15" t="n">
         <v>385</v>
       </c>
-      <c r="D55" s="15" t="n">
-        <v>397</v>
-      </c>
-      <c r="E55" s="15" t="n">
-        <v>407</v>
-      </c>
-      <c r="F55" s="15" t="n">
-        <v>407</v>
-      </c>
-      <c r="G55" s="15" t="n">
-        <v>410</v>
-      </c>
-      <c r="H55" s="15" t="n">
-        <v>410</v>
-      </c>
-      <c r="I55" s="15" t="n">
-        <v>390</v>
-      </c>
-      <c r="J55" s="15" t="n">
-        <v>389</v>
-      </c>
-      <c r="K55" s="15" t="n">
-        <v>388</v>
-      </c>
       <c r="L55" s="15" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="M55" s="15" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="N55" s="15" t="n">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="O55" s="15" t="n">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="P55" s="27">
         <f>SUM(B55:O55)</f>

</xml_diff>